<commit_message>
feat: validate job dependencies
</commit_message>
<xml_diff>
--- a/input/jobs.xlsx
+++ b/input/jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Documents\ControlM-Lab\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{977E4C4E-75C8-4DDB-9197-1BBDCDE000F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A400FE36-1169-46CA-BF61-8AB7DF0665DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{841B3C81-A7A2-42D5-B66D-34338DF1A787}"/>
   </bookViews>
@@ -20,22 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
   <si>
     <t>Job</t>
   </si>
@@ -80,6 +70,57 @@
   </si>
   <si>
     <t>email.sh</t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t>SubApplication</t>
+  </si>
+  <si>
+    <t>RunAs</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>FINANCEIRO</t>
+  </si>
+  <si>
+    <t>IMPORTACAO</t>
+  </si>
+  <si>
+    <t>batch01</t>
+  </si>
+  <si>
+    <t>Recebe arquivos bancários</t>
+  </si>
+  <si>
+    <t>Valida o layout</t>
+  </si>
+  <si>
+    <t>oracle</t>
+  </si>
+  <si>
+    <t>Importa para Oracle</t>
+  </si>
+  <si>
+    <t>RELATORIOS</t>
+  </si>
+  <si>
+    <t>reports</t>
+  </si>
+  <si>
+    <t>Gera relatório</t>
+  </si>
+  <si>
+    <t>Envia e-mail</t>
+  </si>
+  <si>
+    <t>DependsOn</t>
+  </si>
+  <si>
+    <t>JobQueNaoExiste</t>
   </si>
 </sst>
 </file>
@@ -445,73 +486,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0397B0A-4744-41BF-BC40-7FFA2CCFC7A8}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="15.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: validate job dependencies part 2
</commit_message>
<xml_diff>
--- a/input/jobs.xlsx
+++ b/input/jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Documents\ControlM-Lab\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A400FE36-1169-46CA-BF61-8AB7DF0665DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1034C17-7117-4508-9E64-CA309F41C26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{841B3C81-A7A2-42D5-B66D-34338DF1A787}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="33">
   <si>
     <t>Job</t>
   </si>
@@ -120,7 +120,10 @@
     <t>DependsOn</t>
   </si>
   <si>
-    <t>JobQueNaoExiste</t>
+    <t>Folder</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
   </si>
 </sst>
 </file>
@@ -164,13 +167,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,163 +495,185 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0397B0A-4744-41BF-BC40-7FFA2CCFC7A8}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultColWidth="15.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.77734375" style="3"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H4" t="s">
-        <v>31</v>
+      <c r="I4" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>